<commit_message>
Update changes on product stocks, Raw Material, Supplier, Vendor
</commit_message>
<xml_diff>
--- a/ZlaataQA/reports/Extent-Report/Zlaata-QAResults.xlsx
+++ b/ZlaataQA/reports/Extent-Report/Zlaata-QAResults.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="67">
   <si>
     <t>Duration</t>
   </si>
@@ -189,37 +189,55 @@
     <t>device</t>
   </si>
   <si>
-    <t>Aug 06, 2026 11:08:30 AM</t>
-  </si>
-  <si>
-    <t>Aug 06, 2026 11:07:45 AM</t>
-  </si>
-  <si>
-    <t>Aug 06, 2026 11:08:29 AM</t>
-  </si>
-  <si>
-    <t>43.678 s</t>
+    <t>Aug 29, 2026 12:23:11 pm</t>
+  </si>
+  <si>
+    <t>Aug 29, 2026 12:13:33 pm</t>
+  </si>
+  <si>
+    <t>Aug 29, 2026 12:23:09 pm</t>
+  </si>
+  <si>
+    <t>9 m 35.739 s</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>TC_UI_Zlaata_Atbs_01 |Verify admin can add a new Attributes successfully.|"TD_UI_Zlaata_Atbs_01"</t>
-  </si>
-  <si>
-    <t>42.931 s</t>
-  </si>
-  <si>
-    <t>Attributes Management</t>
-  </si>
-  <si>
-    <t>@TC_UI_Zlaata_Atbs_01</t>
-  </si>
-  <si>
-    <t>@Regression</t>
-  </si>
-  <si>
-    <t>42.937 s</t>
+    <t>TC_UI_Zlaata_PS_01 |Verify that stock changes are reflected and saved successfully after adjusting stock.| "TD_UI_Zlaata_PS_01"</t>
+  </si>
+  <si>
+    <t>1 m 59.765 s</t>
+  </si>
+  <si>
+    <t>Product Stock Management</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PS_02 |Verify that stock changes are reflected and saved successfully after adding stock.| "TD_UI_Zlaata_PS_02"</t>
+  </si>
+  <si>
+    <t>4 m 1.222 s</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</t>
+  </si>
+  <si>
+    <t>3 m 34.048 s</t>
+  </si>
+  <si>
+    <t>@TC_UI_Zlaata_PS_01</t>
+  </si>
+  <si>
+    <t>@PS</t>
+  </si>
+  <si>
+    <t>@TC_UI_Zlaata_PS_02</t>
+  </si>
+  <si>
+    <t>@TC_UI_Zlaata_PS_03</t>
+  </si>
+  <si>
+    <t>9 m 35.086 s</t>
   </si>
 </sst>
 </file>
@@ -1787,22 +1805,34 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22</c:f>
+              <c:f>Scenarios!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Atbs_01 |Verify admin can add a new Attributes successfully.|"TD_UI_Zlaata_Atbs_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_01 |Verify that stock changes are reflected and saved successfully after adjusting stock.| "TD_UI_Zlaata_PS_01"</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>TC_UI_Zlaata_PS_02 |Verify that stock changes are reflected and saved successfully after adding stock.| "TD_UI_Zlaata_PS_02"</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$H$22</c:f>
+              <c:f>Scenarios!$H$22:$H$24</c:f>
               <c:numCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>2.0</c:v>
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1859,18 +1889,24 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22</c:f>
+              <c:f>Scenarios!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Atbs_01 |Verify admin can add a new Attributes successfully.|"TD_UI_Zlaata_Atbs_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_01 |Verify that stock changes are reflected and saved successfully after adjusting stock.| "TD_UI_Zlaata_PS_01"</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>TC_UI_Zlaata_PS_02 |Verify that stock changes are reflected and saved successfully after adding stock.| "TD_UI_Zlaata_PS_02"</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$J$22</c:f>
+              <c:f>Scenarios!$J$22:$J$24</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1926,18 +1962,24 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22</c:f>
+              <c:f>Scenarios!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>TC_UI_Zlaata_Atbs_01 |Verify admin can add a new Attributes successfully.|"TD_UI_Zlaata_Atbs_01"</c:v>
+                  <c:v>TC_UI_Zlaata_PS_01 |Verify that stock changes are reflected and saved successfully after adjusting stock.| "TD_UI_Zlaata_PS_01"</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>TC_UI_Zlaata_PS_02 |Verify that stock changes are reflected and saved successfully after adding stock.| "TD_UI_Zlaata_PS_02"</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>TC_UI_Zlaata_PS_03 |Verify that the low stock alert is saved and reflected successfully for the product.| "TD_UI_Zlaata_PS_03"</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$I$22</c:f>
+              <c:f>Scenarios!$I$22:$I$24</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2333,27 +2375,39 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$23</c:f>
+              <c:f>Tags!$B$22:$B$25</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Atbs_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>@TC_UI_Zlaata_PS_02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$D$22:$D$23</c:f>
+              <c:f>Tags!$D$22:$D$25</c:f>
               <c:numCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>1.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.0</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2412,21 +2466,27 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$23</c:f>
+              <c:f>Tags!$B$22:$B$25</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Atbs_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>@TC_UI_Zlaata_PS_02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$F$22:$F$23</c:f>
+              <c:f>Tags!$F$22:$F$25</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2483,21 +2543,27 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$23</c:f>
+              <c:f>Tags!$B$22:$B$25</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>@TC_UI_Zlaata_Atbs_01</c:v>
+                  <c:v>@TC_UI_Zlaata_PS_01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>@Regression</c:v>
+                  <c:v>@PS</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>@TC_UI_Zlaata_PS_02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>@TC_UI_Zlaata_PS_03</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$E$22:$E$23</c:f>
+              <c:f>Tags!$E$22:$E$25</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2706,7 +2772,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Attributes Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2717,7 +2783,7 @@
               <c:numCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1.0</c:v>
+                  <c:v>3.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2778,7 +2844,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Attributes Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2845,7 +2911,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Attributes Management</c:v>
+                  <c:v>Product Stock Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5785,7 +5851,7 @@
     <col min="7" max="7" customWidth="true" width="20.85546875"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="true" password="D119" scenarios="true" objects="true"/>
+  <sheetProtection sheet="true" password="E317" scenarios="true" objects="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -5794,7 +5860,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:J22"/>
+  <dimension ref="B20:J24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.42578125"/>
@@ -5869,13 +5935,63 @@
         <v>29</v>
       </c>
       <c r="G22" s="57" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="H22" s="58" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="I22" s="59"/>
       <c r="J22" s="60"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="54" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="56" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="54" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="57" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="H23" s="58" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="I23" s="59"/>
+      <c r="J23" s="60"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="54" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="54" t="s">
+        <v>57</v>
+      </c>
+      <c r="F24" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="57" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="H24" s="58" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="I24" s="59"/>
+      <c r="J24" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5891,7 +6007,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:I29"/>
+  <dimension ref="B20:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.28515625"/>
@@ -5933,7 +6049,7 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s" s="54">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C22" s="57" t="n">
         <v>1.0</v>
@@ -5949,13 +6065,13 @@
     </row>
     <row r="23">
       <c r="B23" s="54" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C23" s="57" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="D23" s="58" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="E23" s="59"/>
       <c r="F23" s="60"/>
@@ -5963,67 +6079,166 @@
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="35" t="s">
+    <row r="24">
+      <c r="B24" s="54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="57" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="D24" s="58" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="59"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="61" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="57" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="D25" s="58" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="59"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="61" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="49" t="s">
+      <c r="C29" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="36" t="s">
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="35" t="s">
+      <c r="I29" s="35" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="54" t="s">
+    <row r="30">
+      <c r="B30" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="I30" s="55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="I31" s="55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="53"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="62" t="s">
+      <c r="I32" s="55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="53"/>
+      <c r="C33" s="53"/>
+      <c r="D33" s="53"/>
+      <c r="E33" s="53"/>
+      <c r="F33" s="53"/>
+      <c r="G33" s="53"/>
+      <c r="H33" s="62" t="s">
+        <v>60</v>
+      </c>
+      <c r="I33" s="55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="53"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I28" s="55" t="s">
+      <c r="D34" s="53"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="I34" s="55" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="54" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="62" t="s">
+    <row r="35">
+      <c r="B35" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="53"/>
-      <c r="G29" s="53"/>
-      <c r="H29" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I29" s="55" t="s">
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="62" t="s">
+        <v>60</v>
+      </c>
+      <c r="I35" s="55" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
     <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:G33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C35:G35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6114,13 +6329,13 @@
         <v>29</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E22" s="57" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F22" s="58" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G22" s="59"/>
       <c r="H22" s="60"/>
@@ -6128,10 +6343,10 @@
         <v>54</v>
       </c>
       <c r="J22" s="57" t="n">
-        <v>2.0</v>
+        <v>9.0</v>
       </c>
       <c r="K22" s="58" t="n">
-        <v>2.0</v>
+        <v>9.0</v>
       </c>
       <c r="L22" s="59"/>
       <c r="M22" s="60"/>
@@ -6199,13 +6414,13 @@
         <v>9</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>2.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6267,14 +6482,14 @@
       </c>
       <c r="F5" t="n" s="0">
         <f>SUM(F2:F4)</f>
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>21</v>
       </c>
       <c r="H5" t="n" s="0">
         <f>SUM(H2:H4)</f>
-        <v>2.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>